<commit_message>
Export fidelity: remove input-cell shading so finished report is clean
The company template shades all input cells cream (FFFFF3D1) and the Golden Week
block amber (FFFFC000) — the 色付きセル "input here" guide. The surgical-patch
export reproduced this faithfully, so filled reports looked colored/blocky
(consecutive same-value rows read as merged shaded blocks). Rewrote those two
fill definitions to white in assets/template.xlsx.

No structure changed: 379 formulas intact, 50 structural merges intact (activity
Y:AD spans + header merges, same as original), borders/values/fonts unchanged.
Verified in Excel (fill + recalc): clean white form, totals 18/120/15/3 correct.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/template.xlsx
+++ b/assets/template.xlsx
@@ -477,7 +477,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFF3D1"/>
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -489,7 +489,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC000"/>
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>

</xml_diff>

<commit_message>
Fix export: restore borders + decimal number-format + center-align all day rows
Follow-up to the formula-fill: the previously-empty rows had their borders and
decimal number format stripped too, so filled days rendered with missing borders
and time-formatted decimals (8 shown as 0:00, 1.75 as 18:00). Pasted formats from
a complete row onto every day row (borders + 0.00 format) and center-aligned the
data cells (C8:X38, AF8:AF38) per request. Formulas/values/merges unchanged
(473 formulas, 50 merges, 0 shading). Verified in Excel: all rows bordered,
decimals correct, centered, totals correct.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/template.xlsx
+++ b/assets/template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Code - Claude\kinmu-report\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B8E6682B-A8EB-4EA7-8125-F46181F6796D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AC6FC96F-6C1B-497B-898F-995C8455F2B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{D300EFDF-045F-4B6F-92F7-9A5373D84CFD}"/>
+    <workbookView xWindow="1812" yWindow="1812" windowWidth="17280" windowHeight="9420" xr2:uid="{D300EFDF-045F-4B6F-92F7-9A5373D84CFD}"/>
   </bookViews>
   <sheets>
     <sheet name="202602" sheetId="3" r:id="rId1"/>
@@ -468,7 +468,7 @@
       <charset val="128"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -487,14 +487,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="54">
+  <borders count="42">
     <border>
       <left/>
       <right/>
@@ -611,21 +605,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
       <top style="medium">
@@ -645,21 +624,6 @@
         <color indexed="64"/>
       </top>
       <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -696,36 +660,6 @@
       <top style="medium">
         <color indexed="64"/>
       </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
       <bottom style="medium">
         <color indexed="64"/>
       </bottom>
@@ -809,17 +743,6 @@
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -1086,82 +1009,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="126">
+  <cellXfs count="99">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1214,35 +1066,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
@@ -1253,40 +1084,28 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1295,55 +1114,10 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="20" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="1" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="168" fontId="1" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="1" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="1" fillId="2" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="1" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="1" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="1" fillId="2" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="1" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="1" fillId="2" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="1" fillId="2" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="1" fillId="2" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="1" fillId="2" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -1352,191 +1126,188 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" shrinkToFit="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="4" borderId="47" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="4" borderId="48" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="4" borderId="49" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="4" borderId="50" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="4" borderId="51" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="4" borderId="52" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="4" borderId="53" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="42" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="44" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    <xf numFmtId="168" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2104,173 +1875,173 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:32">
-      <c r="AD1" s="37"/>
-      <c r="AE1" s="37" t="s">
+      <c r="AD1" s="26"/>
+      <c r="AE1" s="26" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:32" s="2" customFormat="1" ht="18.75" customHeight="1" thickBot="1">
-      <c r="A2" s="107">
+      <c r="A2" s="60">
         <v>2026</v>
       </c>
-      <c r="B2" s="107"/>
-      <c r="C2" s="68" t="s">
+      <c r="B2" s="60"/>
+      <c r="C2" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="68"/>
-      <c r="E2" s="69">
+      <c r="D2" s="42"/>
+      <c r="E2" s="43">
         <v>5</v>
       </c>
-      <c r="F2" s="68"/>
-      <c r="G2" s="68" t="s">
+      <c r="F2" s="42"/>
+      <c r="G2" s="42" t="s">
         <v>1</v>
       </c>
-      <c r="H2" s="68"/>
-      <c r="I2" s="68"/>
-      <c r="J2" s="68"/>
-      <c r="K2" s="68" t="s">
+      <c r="H2" s="42"/>
+      <c r="I2" s="42"/>
+      <c r="J2" s="42"/>
+      <c r="K2" s="42" t="s">
         <v>2</v>
       </c>
-      <c r="L2" s="32"/>
-      <c r="M2" s="68"/>
-      <c r="O2" s="64" t="s">
+      <c r="L2" s="25"/>
+      <c r="M2" s="42"/>
+      <c r="O2" s="38" t="s">
         <v>30</v>
       </c>
-      <c r="P2" s="95"/>
-      <c r="Q2" s="95"/>
-      <c r="R2" s="95"/>
-      <c r="S2" s="95"/>
-      <c r="T2" s="95"/>
-      <c r="U2" s="95"/>
-      <c r="V2" s="95"/>
-      <c r="W2" s="95"/>
-      <c r="X2" s="95"/>
-      <c r="Z2" s="67" t="s">
+      <c r="P2" s="59"/>
+      <c r="Q2" s="59"/>
+      <c r="R2" s="59"/>
+      <c r="S2" s="59"/>
+      <c r="T2" s="59"/>
+      <c r="U2" s="59"/>
+      <c r="V2" s="59"/>
+      <c r="W2" s="59"/>
+      <c r="X2" s="59"/>
+      <c r="Z2" s="41" t="s">
         <v>24</v>
       </c>
-      <c r="AA2" s="95"/>
-      <c r="AB2" s="95"/>
-      <c r="AC2" s="95"/>
-      <c r="AD2" s="95"/>
-      <c r="AE2" s="95"/>
+      <c r="AA2" s="59"/>
+      <c r="AB2" s="59"/>
+      <c r="AC2" s="59"/>
+      <c r="AD2" s="59"/>
+      <c r="AE2" s="59"/>
     </row>
     <row r="3" spans="1:32" ht="15" thickTop="1">
       <c r="D3" s="2"/>
       <c r="J3" s="15"/>
-      <c r="O3" s="65" t="s">
+      <c r="O3" s="39" t="s">
         <v>25</v>
       </c>
-      <c r="P3" s="95" t="s">
+      <c r="P3" s="59" t="s">
         <v>31</v>
       </c>
-      <c r="Q3" s="95"/>
-      <c r="R3" s="95"/>
-      <c r="S3" s="95"/>
-      <c r="T3" s="95"/>
-      <c r="U3" s="95"/>
-      <c r="V3" s="95"/>
-      <c r="W3" s="95"/>
-      <c r="X3" s="95"/>
-      <c r="Z3" s="67" t="s">
+      <c r="Q3" s="59"/>
+      <c r="R3" s="59"/>
+      <c r="S3" s="59"/>
+      <c r="T3" s="59"/>
+      <c r="U3" s="59"/>
+      <c r="V3" s="59"/>
+      <c r="W3" s="59"/>
+      <c r="X3" s="59"/>
+      <c r="Z3" s="41" t="s">
         <v>23</v>
       </c>
-      <c r="AA3" s="95" t="s">
+      <c r="AA3" s="59" t="s">
         <v>32</v>
       </c>
-      <c r="AB3" s="95"/>
-      <c r="AC3" s="95"/>
-      <c r="AD3" s="95"/>
-      <c r="AE3" s="95"/>
+      <c r="AB3" s="59"/>
+      <c r="AC3" s="59"/>
+      <c r="AD3" s="59"/>
+      <c r="AE3" s="59"/>
     </row>
     <row r="4" spans="1:32" ht="22.5" customHeight="1">
-      <c r="A4" s="105" t="s">
+      <c r="A4" s="88" t="s">
         <v>26</v>
       </c>
-      <c r="B4" s="106"/>
-      <c r="C4" s="66"/>
-      <c r="O4" s="65" t="s">
+      <c r="B4" s="89"/>
+      <c r="C4" s="40"/>
+      <c r="O4" s="39" t="s">
         <v>27</v>
       </c>
-      <c r="P4" s="96"/>
-      <c r="Q4" s="95"/>
-      <c r="R4" s="95"/>
-      <c r="S4" s="95"/>
-      <c r="T4" s="95"/>
-      <c r="U4" s="95"/>
-      <c r="V4" s="95"/>
-      <c r="W4" s="95"/>
-      <c r="X4" s="95"/>
-      <c r="Z4" s="67" t="s">
+      <c r="P4" s="69"/>
+      <c r="Q4" s="59"/>
+      <c r="R4" s="59"/>
+      <c r="S4" s="59"/>
+      <c r="T4" s="59"/>
+      <c r="U4" s="59"/>
+      <c r="V4" s="59"/>
+      <c r="W4" s="59"/>
+      <c r="X4" s="59"/>
+      <c r="Z4" s="41" t="s">
         <v>11</v>
       </c>
-      <c r="AA4" s="94"/>
-      <c r="AB4" s="94"/>
-      <c r="AC4" s="94"/>
-      <c r="AD4" s="94"/>
-      <c r="AE4" s="94"/>
+      <c r="AA4" s="87"/>
+      <c r="AB4" s="87"/>
+      <c r="AC4" s="87"/>
+      <c r="AD4" s="87"/>
+      <c r="AE4" s="87"/>
     </row>
     <row r="5" spans="1:32" ht="9.75" customHeight="1" thickBot="1"/>
     <row r="6" spans="1:32" s="3" customFormat="1" ht="16.5" customHeight="1" thickBot="1">
-      <c r="A6" s="108" t="s">
+      <c r="A6" s="61" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="109"/>
-      <c r="C6" s="85" t="s">
+      <c r="B6" s="62"/>
+      <c r="C6" s="65" t="s">
         <v>20</v>
       </c>
-      <c r="D6" s="112"/>
-      <c r="E6" s="112"/>
-      <c r="F6" s="112"/>
-      <c r="G6" s="112"/>
-      <c r="H6" s="19"/>
-      <c r="I6" s="19"/>
-      <c r="J6" s="19"/>
-      <c r="K6" s="113"/>
-      <c r="L6" s="112"/>
-      <c r="M6" s="112"/>
-      <c r="N6" s="112"/>
-      <c r="O6" s="112"/>
-      <c r="P6" s="85" t="s">
+      <c r="D6" s="66"/>
+      <c r="E6" s="66"/>
+      <c r="F6" s="66"/>
+      <c r="G6" s="66"/>
+      <c r="H6" s="18"/>
+      <c r="I6" s="18"/>
+      <c r="J6" s="18"/>
+      <c r="K6" s="67"/>
+      <c r="L6" s="66"/>
+      <c r="M6" s="66"/>
+      <c r="N6" s="66"/>
+      <c r="O6" s="66"/>
+      <c r="P6" s="65" t="s">
         <v>35</v>
       </c>
-      <c r="Q6" s="112"/>
-      <c r="R6" s="112"/>
-      <c r="S6" s="112"/>
-      <c r="T6" s="112"/>
-      <c r="U6" s="112"/>
-      <c r="V6" s="112"/>
-      <c r="W6" s="114"/>
-      <c r="X6" s="115" t="s">
+      <c r="Q6" s="66"/>
+      <c r="R6" s="66"/>
+      <c r="S6" s="66"/>
+      <c r="T6" s="66"/>
+      <c r="U6" s="66"/>
+      <c r="V6" s="66"/>
+      <c r="W6" s="68"/>
+      <c r="X6" s="78" t="s">
         <v>36</v>
       </c>
-      <c r="Y6" s="97" t="s">
+      <c r="Y6" s="70" t="s">
         <v>33</v>
       </c>
-      <c r="Z6" s="98"/>
-      <c r="AA6" s="98"/>
-      <c r="AB6" s="98"/>
-      <c r="AC6" s="98"/>
-      <c r="AD6" s="99"/>
-      <c r="AE6" s="103" t="s">
+      <c r="Z6" s="71"/>
+      <c r="AA6" s="71"/>
+      <c r="AB6" s="71"/>
+      <c r="AC6" s="71"/>
+      <c r="AD6" s="72"/>
+      <c r="AE6" s="76" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="7" spans="1:32" s="3" customFormat="1" ht="16.5" customHeight="1" thickBot="1">
-      <c r="A7" s="110"/>
-      <c r="B7" s="111"/>
-      <c r="C7" s="42" t="s">
+      <c r="A7" s="63"/>
+      <c r="B7" s="64"/>
+      <c r="C7" s="31" t="s">
         <v>4</v>
       </c>
-      <c r="D7" s="42" t="s">
+      <c r="D7" s="31" t="s">
         <v>4</v>
       </c>
-      <c r="E7" s="43" t="s">
+      <c r="E7" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="F7" s="43" t="s">
+      <c r="F7" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="G7" s="44" t="s">
+      <c r="G7" s="33" t="s">
         <v>12</v>
       </c>
       <c r="H7" s="9" t="s">
@@ -2288,28 +2059,28 @@
       <c r="L7" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="M7" s="20" t="s">
+      <c r="M7" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="N7" s="21" t="s">
+      <c r="N7" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="O7" s="20" t="s">
+      <c r="O7" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="P7" s="73" t="s">
+      <c r="P7" s="47" t="s">
         <v>4</v>
       </c>
-      <c r="Q7" s="42" t="s">
+      <c r="Q7" s="31" t="s">
         <v>4</v>
       </c>
-      <c r="R7" s="44" t="s">
+      <c r="R7" s="33" t="s">
         <v>5</v>
       </c>
-      <c r="S7" s="43" t="s">
+      <c r="S7" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="T7" s="44" t="s">
+      <c r="T7" s="33" t="s">
         <v>12</v>
       </c>
       <c r="U7" s="9" t="s">
@@ -2318,17 +2089,17 @@
       <c r="V7" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="W7" s="74" t="s">
+      <c r="W7" s="48" t="s">
         <v>7</v>
       </c>
-      <c r="X7" s="102"/>
-      <c r="Y7" s="100"/>
-      <c r="Z7" s="101"/>
-      <c r="AA7" s="101"/>
-      <c r="AB7" s="101"/>
-      <c r="AC7" s="101"/>
-      <c r="AD7" s="102"/>
-      <c r="AE7" s="104"/>
+      <c r="X7" s="75"/>
+      <c r="Y7" s="73"/>
+      <c r="Z7" s="74"/>
+      <c r="AA7" s="74"/>
+      <c r="AB7" s="74"/>
+      <c r="AC7" s="74"/>
+      <c r="AD7" s="75"/>
+      <c r="AE7" s="77"/>
     </row>
     <row r="8" spans="1:32" ht="18" customHeight="1" thickBot="1">
       <c r="A8" s="6">
@@ -2339,16 +2110,16 @@
         <f>A8</f>
         <v>46143</v>
       </c>
-      <c r="C8" s="48"/>
-      <c r="D8" s="45"/>
-      <c r="E8" s="49"/>
-      <c r="F8" s="46"/>
-      <c r="G8" s="50"/>
-      <c r="H8" s="24" t="str">
+      <c r="C8" s="91"/>
+      <c r="D8" s="92"/>
+      <c r="E8" s="34"/>
+      <c r="F8" s="93"/>
+      <c r="G8" s="34"/>
+      <c r="H8" s="94" t="str">
         <f t="shared" ref="H8:H38" si="0">IF(G8="","",G8/"01:00:00")</f>
         <v/>
       </c>
-      <c r="I8" s="25" t="str">
+      <c r="I8" s="95" t="str">
         <f t="shared" ref="I8:I38" si="1">IF(C8="","",E8-C8-G8)</f>
         <v/>
       </c>
@@ -2356,7 +2127,7 @@
         <f t="shared" ref="J8:J38" si="2">IF(I8="","",IF(I8&gt;$C$46,$C$46,I8))</f>
         <v/>
       </c>
-      <c r="K8" s="24" t="str">
+      <c r="K8" s="94" t="str">
         <f t="shared" ref="K8:K38" si="3">IF(J8="","",J8/"01:00:00")</f>
         <v/>
       </c>
@@ -2364,7 +2135,7 @@
         <f t="shared" ref="L8:L38" si="4">IF(OR(I8&lt;=$C$46,I8=""),"",I8-J8-N8)</f>
         <v/>
       </c>
-      <c r="M8" s="24" t="str">
+      <c r="M8" s="94" t="str">
         <f t="shared" ref="M8:M38" si="5">IF(L8="","",L8/"01:00:00")</f>
         <v/>
       </c>
@@ -2372,36 +2143,36 @@
         <f t="shared" ref="N8:N38" si="6">5/24-MIN(C8,5/24)+MAX((E8&lt;C8)+E8,22/24)-22/24</f>
         <v>0</v>
       </c>
-      <c r="O8" s="33" t="str">
+      <c r="O8" s="96" t="str">
         <f t="shared" ref="O8:O38" si="7">IF(M8="","",N8/"01:00:00")</f>
         <v/>
       </c>
-      <c r="P8" s="54"/>
-      <c r="Q8" s="55"/>
-      <c r="R8" s="56"/>
-      <c r="S8" s="55"/>
-      <c r="T8" s="47"/>
-      <c r="U8" s="22" t="str">
+      <c r="P8" s="91"/>
+      <c r="Q8" s="97"/>
+      <c r="R8" s="34"/>
+      <c r="S8" s="97"/>
+      <c r="T8" s="34"/>
+      <c r="U8" s="94" t="str">
         <f t="shared" ref="U8:U38" si="8">IF(T8="","",T8/"01:00:00")</f>
         <v/>
       </c>
-      <c r="V8" s="23" t="str">
+      <c r="V8" s="95" t="str">
         <f t="shared" ref="V8:V38" si="9">IF(P8="","",R8-P8-T8)</f>
         <v/>
       </c>
-      <c r="W8" s="34" t="str">
+      <c r="W8" s="98" t="str">
         <f t="shared" ref="W8:W38" si="10">IF(V8="","",V8/"01:00:00")</f>
         <v/>
       </c>
-      <c r="X8" s="59"/>
-      <c r="Y8" s="116"/>
-      <c r="Z8" s="117"/>
-      <c r="AA8" s="117"/>
-      <c r="AB8" s="117"/>
-      <c r="AC8" s="117"/>
-      <c r="AD8" s="118"/>
-      <c r="AE8" s="70"/>
-      <c r="AF8" s="1" t="str">
+      <c r="X8" s="35"/>
+      <c r="Y8" s="50"/>
+      <c r="Z8" s="51"/>
+      <c r="AA8" s="51"/>
+      <c r="AB8" s="51"/>
+      <c r="AC8" s="51"/>
+      <c r="AD8" s="52"/>
+      <c r="AE8" s="44"/>
+      <c r="AF8" s="3" t="str">
         <f t="shared" ref="AF8:AF38" si="11">IF(AND(B8&lt;&gt;"土",B8&lt;&gt;"日",OR(AND(C8&gt;0,C8&lt;24),X8&gt;0)),"稼働日","")</f>
         <v/>
       </c>
@@ -2415,69 +2186,69 @@
         <f>A9</f>
         <v>46144</v>
       </c>
-      <c r="C9" s="76"/>
-      <c r="D9" s="77"/>
-      <c r="E9" s="77"/>
-      <c r="F9" s="77"/>
-      <c r="G9" s="77"/>
-      <c r="H9" s="77" t="str">
+      <c r="C9" s="91"/>
+      <c r="D9" s="92"/>
+      <c r="E9" s="34"/>
+      <c r="F9" s="93"/>
+      <c r="G9" s="34"/>
+      <c r="H9" s="94" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="I9" s="77" t="str">
+      <c r="I9" s="95" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J9" s="77" t="str">
+      <c r="J9" s="8" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K9" s="77" t="str">
+      <c r="K9" s="94" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="L9" s="77" t="str">
+      <c r="L9" s="8" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="M9" s="77" t="str">
+      <c r="M9" s="94" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="N9" s="77">
+      <c r="N9" s="8">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="O9" s="78" t="str">
+      <c r="O9" s="96" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="P9" s="48"/>
-      <c r="Q9" s="57"/>
-      <c r="R9" s="49"/>
-      <c r="S9" s="57"/>
-      <c r="T9" s="50"/>
-      <c r="U9" s="24" t="str">
+      <c r="P9" s="91"/>
+      <c r="Q9" s="97"/>
+      <c r="R9" s="34"/>
+      <c r="S9" s="97"/>
+      <c r="T9" s="34"/>
+      <c r="U9" s="94" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="V9" s="25" t="str">
+      <c r="V9" s="95" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="W9" s="35" t="str">
+      <c r="W9" s="98" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="X9" s="60"/>
-      <c r="Y9" s="116"/>
-      <c r="Z9" s="117"/>
-      <c r="AA9" s="117"/>
-      <c r="AB9" s="117"/>
-      <c r="AC9" s="117"/>
-      <c r="AD9" s="118"/>
-      <c r="AE9" s="71"/>
-      <c r="AF9" s="1" t="str">
+      <c r="X9" s="35"/>
+      <c r="Y9" s="50"/>
+      <c r="Z9" s="51"/>
+      <c r="AA9" s="51"/>
+      <c r="AB9" s="51"/>
+      <c r="AC9" s="51"/>
+      <c r="AD9" s="52"/>
+      <c r="AE9" s="45"/>
+      <c r="AF9" s="3" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
@@ -2491,69 +2262,69 @@
         <f t="shared" ref="B10:B38" si="12">A10</f>
         <v>46145</v>
       </c>
-      <c r="C10" s="79"/>
-      <c r="D10" s="80"/>
-      <c r="E10" s="80"/>
-      <c r="F10" s="80"/>
-      <c r="G10" s="80"/>
-      <c r="H10" s="80" t="str">
+      <c r="C10" s="91"/>
+      <c r="D10" s="92"/>
+      <c r="E10" s="34"/>
+      <c r="F10" s="93"/>
+      <c r="G10" s="34"/>
+      <c r="H10" s="94" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="I10" s="80" t="str">
+      <c r="I10" s="95" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J10" s="80" t="str">
+      <c r="J10" s="8" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K10" s="80" t="str">
+      <c r="K10" s="94" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="L10" s="80" t="str">
+      <c r="L10" s="8" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="M10" s="80" t="str">
+      <c r="M10" s="94" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="N10" s="80">
+      <c r="N10" s="8">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="O10" s="81" t="str">
+      <c r="O10" s="96" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="P10" s="48"/>
-      <c r="Q10" s="57"/>
-      <c r="R10" s="49"/>
-      <c r="S10" s="57"/>
-      <c r="T10" s="50"/>
-      <c r="U10" s="24" t="str">
+      <c r="P10" s="91"/>
+      <c r="Q10" s="97"/>
+      <c r="R10" s="34"/>
+      <c r="S10" s="97"/>
+      <c r="T10" s="34"/>
+      <c r="U10" s="94" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="V10" s="25" t="str">
+      <c r="V10" s="95" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="W10" s="35" t="str">
+      <c r="W10" s="98" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="X10" s="60"/>
-      <c r="Y10" s="116"/>
-      <c r="Z10" s="117"/>
-      <c r="AA10" s="117"/>
-      <c r="AB10" s="117"/>
-      <c r="AC10" s="117"/>
-      <c r="AD10" s="118"/>
-      <c r="AE10" s="71"/>
-      <c r="AF10" s="1" t="str">
+      <c r="X10" s="35"/>
+      <c r="Y10" s="50"/>
+      <c r="Z10" s="51"/>
+      <c r="AA10" s="51"/>
+      <c r="AB10" s="51"/>
+      <c r="AC10" s="51"/>
+      <c r="AD10" s="52"/>
+      <c r="AE10" s="45"/>
+      <c r="AF10" s="3" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
@@ -2567,69 +2338,69 @@
         <f t="shared" si="12"/>
         <v>46146</v>
       </c>
-      <c r="C11" s="79"/>
-      <c r="D11" s="80"/>
-      <c r="E11" s="80"/>
-      <c r="F11" s="80"/>
-      <c r="G11" s="80"/>
-      <c r="H11" s="80" t="str">
+      <c r="C11" s="91"/>
+      <c r="D11" s="92"/>
+      <c r="E11" s="34"/>
+      <c r="F11" s="93"/>
+      <c r="G11" s="34"/>
+      <c r="H11" s="94" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="I11" s="80" t="str">
+      <c r="I11" s="95" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J11" s="80" t="str">
+      <c r="J11" s="8" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K11" s="80" t="str">
+      <c r="K11" s="94" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="L11" s="80" t="str">
+      <c r="L11" s="8" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="M11" s="80" t="str">
+      <c r="M11" s="94" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="N11" s="80">
+      <c r="N11" s="8">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="O11" s="81" t="str">
+      <c r="O11" s="96" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="P11" s="48"/>
-      <c r="Q11" s="57"/>
-      <c r="R11" s="49"/>
-      <c r="S11" s="57"/>
-      <c r="T11" s="50"/>
-      <c r="U11" s="24" t="str">
+      <c r="P11" s="91"/>
+      <c r="Q11" s="97"/>
+      <c r="R11" s="34"/>
+      <c r="S11" s="97"/>
+      <c r="T11" s="34"/>
+      <c r="U11" s="94" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="V11" s="25" t="str">
+      <c r="V11" s="95" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="W11" s="35" t="str">
+      <c r="W11" s="98" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="X11" s="60"/>
-      <c r="Y11" s="119"/>
-      <c r="Z11" s="120"/>
-      <c r="AA11" s="120"/>
-      <c r="AB11" s="120"/>
-      <c r="AC11" s="120"/>
-      <c r="AD11" s="121"/>
-      <c r="AE11" s="71"/>
-      <c r="AF11" s="1" t="str">
+      <c r="X11" s="35"/>
+      <c r="Y11" s="90"/>
+      <c r="Z11" s="57"/>
+      <c r="AA11" s="57"/>
+      <c r="AB11" s="57"/>
+      <c r="AC11" s="57"/>
+      <c r="AD11" s="58"/>
+      <c r="AE11" s="45"/>
+      <c r="AF11" s="3" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
@@ -2643,69 +2414,69 @@
         <f t="shared" si="12"/>
         <v>46147</v>
       </c>
-      <c r="C12" s="79"/>
-      <c r="D12" s="80"/>
-      <c r="E12" s="80"/>
-      <c r="F12" s="80"/>
-      <c r="G12" s="80"/>
-      <c r="H12" s="80" t="str">
+      <c r="C12" s="91"/>
+      <c r="D12" s="92"/>
+      <c r="E12" s="34"/>
+      <c r="F12" s="93"/>
+      <c r="G12" s="34"/>
+      <c r="H12" s="94" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="I12" s="80" t="str">
+      <c r="I12" s="95" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J12" s="80" t="str">
+      <c r="J12" s="8" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K12" s="80" t="str">
+      <c r="K12" s="94" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="L12" s="80" t="str">
+      <c r="L12" s="8" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="M12" s="80" t="str">
+      <c r="M12" s="94" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="N12" s="80">
+      <c r="N12" s="8">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="O12" s="81" t="str">
+      <c r="O12" s="96" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="P12" s="48"/>
-      <c r="Q12" s="57"/>
-      <c r="R12" s="49"/>
-      <c r="S12" s="57"/>
-      <c r="T12" s="50"/>
-      <c r="U12" s="24" t="str">
+      <c r="P12" s="91"/>
+      <c r="Q12" s="97"/>
+      <c r="R12" s="34"/>
+      <c r="S12" s="97"/>
+      <c r="T12" s="34"/>
+      <c r="U12" s="94" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="V12" s="25" t="str">
+      <c r="V12" s="95" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="W12" s="35" t="str">
+      <c r="W12" s="98" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="X12" s="60"/>
-      <c r="Y12" s="119"/>
-      <c r="Z12" s="120"/>
-      <c r="AA12" s="120"/>
-      <c r="AB12" s="120"/>
-      <c r="AC12" s="120"/>
-      <c r="AD12" s="121"/>
-      <c r="AE12" s="71"/>
-      <c r="AF12" s="1" t="str">
+      <c r="X12" s="35"/>
+      <c r="Y12" s="90"/>
+      <c r="Z12" s="57"/>
+      <c r="AA12" s="57"/>
+      <c r="AB12" s="57"/>
+      <c r="AC12" s="57"/>
+      <c r="AD12" s="58"/>
+      <c r="AE12" s="45"/>
+      <c r="AF12" s="3" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
@@ -2719,69 +2490,69 @@
         <f t="shared" si="12"/>
         <v>46148</v>
       </c>
-      <c r="C13" s="82"/>
-      <c r="D13" s="83"/>
-      <c r="E13" s="83"/>
-      <c r="F13" s="83"/>
-      <c r="G13" s="83"/>
-      <c r="H13" s="83" t="str">
+      <c r="C13" s="91"/>
+      <c r="D13" s="92"/>
+      <c r="E13" s="34"/>
+      <c r="F13" s="93"/>
+      <c r="G13" s="34"/>
+      <c r="H13" s="94" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="I13" s="83" t="str">
+      <c r="I13" s="95" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J13" s="83" t="str">
+      <c r="J13" s="8" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K13" s="83" t="str">
+      <c r="K13" s="94" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="L13" s="83" t="str">
+      <c r="L13" s="8" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="M13" s="83" t="str">
+      <c r="M13" s="94" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="N13" s="83">
+      <c r="N13" s="8">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="O13" s="84" t="str">
+      <c r="O13" s="96" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="P13" s="48"/>
-      <c r="Q13" s="57"/>
-      <c r="R13" s="49"/>
-      <c r="S13" s="57"/>
-      <c r="T13" s="50"/>
-      <c r="U13" s="24" t="str">
+      <c r="P13" s="91"/>
+      <c r="Q13" s="97"/>
+      <c r="R13" s="34"/>
+      <c r="S13" s="97"/>
+      <c r="T13" s="34"/>
+      <c r="U13" s="94" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="V13" s="25" t="str">
+      <c r="V13" s="95" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="W13" s="35" t="str">
+      <c r="W13" s="98" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="X13" s="60"/>
-      <c r="Y13" s="116"/>
-      <c r="Z13" s="117"/>
-      <c r="AA13" s="117"/>
-      <c r="AB13" s="117"/>
-      <c r="AC13" s="117"/>
-      <c r="AD13" s="118"/>
-      <c r="AE13" s="71"/>
-      <c r="AF13" s="1" t="str">
+      <c r="X13" s="35"/>
+      <c r="Y13" s="50"/>
+      <c r="Z13" s="51"/>
+      <c r="AA13" s="51"/>
+      <c r="AB13" s="51"/>
+      <c r="AC13" s="51"/>
+      <c r="AD13" s="52"/>
+      <c r="AE13" s="45"/>
+      <c r="AF13" s="3" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
@@ -2795,16 +2566,16 @@
         <f t="shared" si="12"/>
         <v>46149</v>
       </c>
-      <c r="C14" s="48"/>
-      <c r="D14" s="45"/>
-      <c r="E14" s="49"/>
-      <c r="F14" s="46"/>
-      <c r="G14" s="50"/>
-      <c r="H14" s="24" t="str">
+      <c r="C14" s="91"/>
+      <c r="D14" s="92"/>
+      <c r="E14" s="34"/>
+      <c r="F14" s="93"/>
+      <c r="G14" s="34"/>
+      <c r="H14" s="94" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="I14" s="25" t="str">
+      <c r="I14" s="95" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -2812,7 +2583,7 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K14" s="24" t="str">
+      <c r="K14" s="94" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -2820,7 +2591,7 @@
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="M14" s="24" t="str">
+      <c r="M14" s="94" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -2828,36 +2599,36 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="O14" s="33" t="str">
+      <c r="O14" s="96" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="P14" s="48"/>
-      <c r="Q14" s="57"/>
-      <c r="R14" s="49"/>
-      <c r="S14" s="57"/>
-      <c r="T14" s="50"/>
-      <c r="U14" s="24" t="str">
+      <c r="P14" s="91"/>
+      <c r="Q14" s="97"/>
+      <c r="R14" s="34"/>
+      <c r="S14" s="97"/>
+      <c r="T14" s="34"/>
+      <c r="U14" s="94" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="V14" s="25" t="str">
+      <c r="V14" s="95" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="W14" s="35" t="str">
+      <c r="W14" s="98" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="X14" s="60"/>
-      <c r="Y14" s="116"/>
-      <c r="Z14" s="117"/>
-      <c r="AA14" s="117"/>
-      <c r="AB14" s="117"/>
-      <c r="AC14" s="117"/>
-      <c r="AD14" s="118"/>
-      <c r="AE14" s="71"/>
-      <c r="AF14" s="1" t="str">
+      <c r="X14" s="35"/>
+      <c r="Y14" s="50"/>
+      <c r="Z14" s="51"/>
+      <c r="AA14" s="51"/>
+      <c r="AB14" s="51"/>
+      <c r="AC14" s="51"/>
+      <c r="AD14" s="52"/>
+      <c r="AE14" s="45"/>
+      <c r="AF14" s="3" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
@@ -2871,16 +2642,16 @@
         <f t="shared" si="12"/>
         <v>46150</v>
       </c>
-      <c r="C15" s="48"/>
-      <c r="D15" s="45"/>
-      <c r="E15" s="49"/>
-      <c r="F15" s="46"/>
-      <c r="G15" s="50"/>
-      <c r="H15" s="24" t="str">
+      <c r="C15" s="91"/>
+      <c r="D15" s="92"/>
+      <c r="E15" s="34"/>
+      <c r="F15" s="93"/>
+      <c r="G15" s="34"/>
+      <c r="H15" s="94" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="I15" s="25" t="str">
+      <c r="I15" s="95" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -2888,7 +2659,7 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K15" s="24" t="str">
+      <c r="K15" s="94" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -2896,7 +2667,7 @@
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="M15" s="24" t="str">
+      <c r="M15" s="94" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -2904,36 +2675,36 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="O15" s="33" t="str">
+      <c r="O15" s="96" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="P15" s="48"/>
-      <c r="Q15" s="57"/>
-      <c r="R15" s="49"/>
-      <c r="S15" s="57"/>
-      <c r="T15" s="50"/>
-      <c r="U15" s="24" t="str">
+      <c r="P15" s="91"/>
+      <c r="Q15" s="97"/>
+      <c r="R15" s="34"/>
+      <c r="S15" s="97"/>
+      <c r="T15" s="34"/>
+      <c r="U15" s="94" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="V15" s="25" t="str">
+      <c r="V15" s="95" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="W15" s="35" t="str">
+      <c r="W15" s="98" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="X15" s="60"/>
-      <c r="Y15" s="116"/>
-      <c r="Z15" s="117"/>
-      <c r="AA15" s="117"/>
-      <c r="AB15" s="117"/>
-      <c r="AC15" s="117"/>
-      <c r="AD15" s="118"/>
-      <c r="AE15" s="71"/>
-      <c r="AF15" s="1" t="str">
+      <c r="X15" s="35"/>
+      <c r="Y15" s="50"/>
+      <c r="Z15" s="51"/>
+      <c r="AA15" s="51"/>
+      <c r="AB15" s="51"/>
+      <c r="AC15" s="51"/>
+      <c r="AD15" s="52"/>
+      <c r="AE15" s="45"/>
+      <c r="AF15" s="3" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
@@ -2947,16 +2718,16 @@
         <f t="shared" si="12"/>
         <v>46151</v>
       </c>
-      <c r="C16" s="48"/>
-      <c r="D16" s="45"/>
-      <c r="E16" s="49"/>
-      <c r="F16" s="46"/>
-      <c r="G16" s="50"/>
-      <c r="H16" s="24" t="str">
+      <c r="C16" s="91"/>
+      <c r="D16" s="92"/>
+      <c r="E16" s="34"/>
+      <c r="F16" s="93"/>
+      <c r="G16" s="34"/>
+      <c r="H16" s="94" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="I16" s="25" t="str">
+      <c r="I16" s="95" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -2964,7 +2735,7 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K16" s="24" t="str">
+      <c r="K16" s="94" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -2972,7 +2743,7 @@
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="M16" s="24" t="str">
+      <c r="M16" s="94" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -2980,42 +2751,42 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="O16" s="33" t="str">
+      <c r="O16" s="96" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="P16" s="48"/>
-      <c r="Q16" s="57" t="str">
+      <c r="P16" s="91"/>
+      <c r="Q16" s="97" t="str">
         <f t="shared" ref="Q16:Q38" si="14">IF(P16="","",P16/"01:00:00")</f>
         <v/>
       </c>
-      <c r="R16" s="49"/>
-      <c r="S16" s="57" t="str">
+      <c r="R16" s="34"/>
+      <c r="S16" s="97" t="str">
         <f t="shared" ref="S16:S38" si="15">IF(R16="","",R16/"01:00:00")</f>
         <v/>
       </c>
-      <c r="T16" s="50"/>
-      <c r="U16" s="24" t="str">
+      <c r="T16" s="34"/>
+      <c r="U16" s="94" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="V16" s="25" t="str">
+      <c r="V16" s="95" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="W16" s="35" t="str">
+      <c r="W16" s="98" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="X16" s="60"/>
-      <c r="Y16" s="116"/>
-      <c r="Z16" s="117"/>
-      <c r="AA16" s="117"/>
-      <c r="AB16" s="117"/>
-      <c r="AC16" s="117"/>
-      <c r="AD16" s="118"/>
-      <c r="AE16" s="71"/>
-      <c r="AF16" s="1" t="str">
+      <c r="X16" s="35"/>
+      <c r="Y16" s="50"/>
+      <c r="Z16" s="51"/>
+      <c r="AA16" s="51"/>
+      <c r="AB16" s="51"/>
+      <c r="AC16" s="51"/>
+      <c r="AD16" s="52"/>
+      <c r="AE16" s="45"/>
+      <c r="AF16" s="3" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
@@ -3029,16 +2800,16 @@
         <f t="shared" si="12"/>
         <v>46152</v>
       </c>
-      <c r="C17" s="48"/>
-      <c r="D17" s="45"/>
-      <c r="E17" s="49"/>
-      <c r="F17" s="46"/>
-      <c r="G17" s="50"/>
-      <c r="H17" s="24" t="str">
+      <c r="C17" s="91"/>
+      <c r="D17" s="92"/>
+      <c r="E17" s="34"/>
+      <c r="F17" s="93"/>
+      <c r="G17" s="34"/>
+      <c r="H17" s="94" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="I17" s="25" t="str">
+      <c r="I17" s="95" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -3046,7 +2817,7 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K17" s="24" t="str">
+      <c r="K17" s="94" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -3054,7 +2825,7 @@
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="M17" s="24" t="str">
+      <c r="M17" s="94" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -3062,42 +2833,42 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="O17" s="33" t="str">
+      <c r="O17" s="96" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="P17" s="48"/>
-      <c r="Q17" s="57" t="str">
+      <c r="P17" s="91"/>
+      <c r="Q17" s="97" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="R17" s="49"/>
-      <c r="S17" s="57" t="str">
+      <c r="R17" s="34"/>
+      <c r="S17" s="97" t="str">
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="T17" s="50"/>
-      <c r="U17" s="24" t="str">
+      <c r="T17" s="34"/>
+      <c r="U17" s="94" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="V17" s="25" t="str">
+      <c r="V17" s="95" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="W17" s="35" t="str">
+      <c r="W17" s="98" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="X17" s="60"/>
-      <c r="Y17" s="116"/>
-      <c r="Z17" s="117"/>
-      <c r="AA17" s="117"/>
-      <c r="AB17" s="117"/>
-      <c r="AC17" s="117"/>
-      <c r="AD17" s="118"/>
-      <c r="AE17" s="71"/>
-      <c r="AF17" s="1" t="str">
+      <c r="X17" s="35"/>
+      <c r="Y17" s="50"/>
+      <c r="Z17" s="51"/>
+      <c r="AA17" s="51"/>
+      <c r="AB17" s="51"/>
+      <c r="AC17" s="51"/>
+      <c r="AD17" s="52"/>
+      <c r="AE17" s="45"/>
+      <c r="AF17" s="3" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
@@ -3111,16 +2882,16 @@
         <f t="shared" si="12"/>
         <v>46153</v>
       </c>
-      <c r="C18" s="48"/>
-      <c r="D18" s="45"/>
-      <c r="E18" s="49"/>
-      <c r="F18" s="46"/>
-      <c r="G18" s="50"/>
-      <c r="H18" s="24" t="str">
+      <c r="C18" s="91"/>
+      <c r="D18" s="92"/>
+      <c r="E18" s="34"/>
+      <c r="F18" s="93"/>
+      <c r="G18" s="34"/>
+      <c r="H18" s="94" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="I18" s="25" t="str">
+      <c r="I18" s="95" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -3128,7 +2899,7 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K18" s="24" t="str">
+      <c r="K18" s="94" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -3136,7 +2907,7 @@
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="M18" s="24" t="str">
+      <c r="M18" s="94" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -3144,42 +2915,42 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="O18" s="33" t="str">
+      <c r="O18" s="96" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="P18" s="48"/>
-      <c r="Q18" s="57" t="str">
+      <c r="P18" s="91"/>
+      <c r="Q18" s="97" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="R18" s="49"/>
-      <c r="S18" s="57" t="str">
+      <c r="R18" s="34"/>
+      <c r="S18" s="97" t="str">
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="T18" s="50"/>
-      <c r="U18" s="24" t="str">
+      <c r="T18" s="34"/>
+      <c r="U18" s="94" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="V18" s="25" t="str">
+      <c r="V18" s="95" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="W18" s="35" t="str">
+      <c r="W18" s="98" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="X18" s="60"/>
-      <c r="Y18" s="116"/>
-      <c r="Z18" s="117"/>
-      <c r="AA18" s="117"/>
-      <c r="AB18" s="117"/>
-      <c r="AC18" s="117"/>
-      <c r="AD18" s="118"/>
-      <c r="AE18" s="71"/>
-      <c r="AF18" s="1" t="str">
+      <c r="X18" s="35"/>
+      <c r="Y18" s="50"/>
+      <c r="Z18" s="51"/>
+      <c r="AA18" s="51"/>
+      <c r="AB18" s="51"/>
+      <c r="AC18" s="51"/>
+      <c r="AD18" s="52"/>
+      <c r="AE18" s="45"/>
+      <c r="AF18" s="3" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
@@ -3193,16 +2964,16 @@
         <f t="shared" si="12"/>
         <v>46154</v>
       </c>
-      <c r="C19" s="48"/>
-      <c r="D19" s="45"/>
-      <c r="E19" s="49"/>
-      <c r="F19" s="46"/>
-      <c r="G19" s="50"/>
-      <c r="H19" s="24" t="str">
+      <c r="C19" s="91"/>
+      <c r="D19" s="92"/>
+      <c r="E19" s="34"/>
+      <c r="F19" s="93"/>
+      <c r="G19" s="34"/>
+      <c r="H19" s="94" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="I19" s="25" t="str">
+      <c r="I19" s="95" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -3210,7 +2981,7 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K19" s="24" t="str">
+      <c r="K19" s="94" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -3218,7 +2989,7 @@
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="M19" s="24" t="str">
+      <c r="M19" s="94" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -3226,42 +2997,42 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="O19" s="33" t="str">
+      <c r="O19" s="96" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="P19" s="48"/>
-      <c r="Q19" s="57" t="str">
+      <c r="P19" s="91"/>
+      <c r="Q19" s="97" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="R19" s="49"/>
-      <c r="S19" s="57" t="str">
+      <c r="R19" s="34"/>
+      <c r="S19" s="97" t="str">
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="T19" s="50"/>
-      <c r="U19" s="24" t="str">
+      <c r="T19" s="34"/>
+      <c r="U19" s="94" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="V19" s="25" t="str">
+      <c r="V19" s="95" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="W19" s="35" t="str">
+      <c r="W19" s="98" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="X19" s="60"/>
-      <c r="Y19" s="116"/>
-      <c r="Z19" s="117"/>
-      <c r="AA19" s="117"/>
-      <c r="AB19" s="117"/>
-      <c r="AC19" s="117"/>
-      <c r="AD19" s="118"/>
-      <c r="AE19" s="71"/>
-      <c r="AF19" s="1" t="str">
+      <c r="X19" s="35"/>
+      <c r="Y19" s="50"/>
+      <c r="Z19" s="51"/>
+      <c r="AA19" s="51"/>
+      <c r="AB19" s="51"/>
+      <c r="AC19" s="51"/>
+      <c r="AD19" s="52"/>
+      <c r="AE19" s="45"/>
+      <c r="AF19" s="3" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
@@ -3275,16 +3046,16 @@
         <f t="shared" si="12"/>
         <v>46155</v>
       </c>
-      <c r="C20" s="48"/>
-      <c r="D20" s="45"/>
-      <c r="E20" s="49"/>
-      <c r="F20" s="46"/>
-      <c r="G20" s="50"/>
-      <c r="H20" s="24" t="str">
+      <c r="C20" s="91"/>
+      <c r="D20" s="92"/>
+      <c r="E20" s="34"/>
+      <c r="F20" s="93"/>
+      <c r="G20" s="34"/>
+      <c r="H20" s="94" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="I20" s="25" t="str">
+      <c r="I20" s="95" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -3292,7 +3063,7 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K20" s="24" t="str">
+      <c r="K20" s="94" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -3300,7 +3071,7 @@
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="M20" s="24" t="str">
+      <c r="M20" s="94" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -3308,42 +3079,42 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="O20" s="33" t="str">
+      <c r="O20" s="96" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="P20" s="48"/>
-      <c r="Q20" s="57" t="str">
+      <c r="P20" s="91"/>
+      <c r="Q20" s="97" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="R20" s="49"/>
-      <c r="S20" s="57" t="str">
+      <c r="R20" s="34"/>
+      <c r="S20" s="97" t="str">
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="T20" s="50"/>
-      <c r="U20" s="24" t="str">
+      <c r="T20" s="34"/>
+      <c r="U20" s="94" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="V20" s="25" t="str">
+      <c r="V20" s="95" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="W20" s="35" t="str">
+      <c r="W20" s="98" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="X20" s="60"/>
-      <c r="Y20" s="116"/>
-      <c r="Z20" s="117"/>
-      <c r="AA20" s="117"/>
-      <c r="AB20" s="117"/>
-      <c r="AC20" s="117"/>
-      <c r="AD20" s="118"/>
-      <c r="AE20" s="71"/>
-      <c r="AF20" s="1" t="str">
+      <c r="X20" s="35"/>
+      <c r="Y20" s="50"/>
+      <c r="Z20" s="51"/>
+      <c r="AA20" s="51"/>
+      <c r="AB20" s="51"/>
+      <c r="AC20" s="51"/>
+      <c r="AD20" s="52"/>
+      <c r="AE20" s="45"/>
+      <c r="AF20" s="3" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
@@ -3357,16 +3128,16 @@
         <f t="shared" si="12"/>
         <v>46156</v>
       </c>
-      <c r="C21" s="48"/>
-      <c r="D21" s="45"/>
-      <c r="E21" s="49"/>
-      <c r="F21" s="46"/>
-      <c r="G21" s="50"/>
-      <c r="H21" s="24" t="str">
+      <c r="C21" s="91"/>
+      <c r="D21" s="92"/>
+      <c r="E21" s="34"/>
+      <c r="F21" s="93"/>
+      <c r="G21" s="34"/>
+      <c r="H21" s="94" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="I21" s="25" t="str">
+      <c r="I21" s="95" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -3374,7 +3145,7 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K21" s="24" t="str">
+      <c r="K21" s="94" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -3382,7 +3153,7 @@
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="M21" s="24" t="str">
+      <c r="M21" s="94" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -3390,42 +3161,42 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="O21" s="33" t="str">
+      <c r="O21" s="96" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="P21" s="48"/>
-      <c r="Q21" s="57" t="str">
+      <c r="P21" s="91"/>
+      <c r="Q21" s="97" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="R21" s="49"/>
-      <c r="S21" s="57" t="str">
+      <c r="R21" s="34"/>
+      <c r="S21" s="97" t="str">
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="T21" s="50"/>
-      <c r="U21" s="24" t="str">
+      <c r="T21" s="34"/>
+      <c r="U21" s="94" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="V21" s="25" t="str">
+      <c r="V21" s="95" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="W21" s="35" t="str">
+      <c r="W21" s="98" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="X21" s="60"/>
-      <c r="Y21" s="116"/>
-      <c r="Z21" s="117"/>
-      <c r="AA21" s="117"/>
-      <c r="AB21" s="117"/>
-      <c r="AC21" s="117"/>
-      <c r="AD21" s="118"/>
-      <c r="AE21" s="71"/>
-      <c r="AF21" s="1" t="str">
+      <c r="X21" s="35"/>
+      <c r="Y21" s="50"/>
+      <c r="Z21" s="51"/>
+      <c r="AA21" s="51"/>
+      <c r="AB21" s="51"/>
+      <c r="AC21" s="51"/>
+      <c r="AD21" s="52"/>
+      <c r="AE21" s="45"/>
+      <c r="AF21" s="3" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
@@ -3439,16 +3210,16 @@
         <f t="shared" si="12"/>
         <v>46157</v>
       </c>
-      <c r="C22" s="48"/>
-      <c r="D22" s="45"/>
-      <c r="E22" s="49"/>
-      <c r="F22" s="46"/>
-      <c r="G22" s="50"/>
-      <c r="H22" s="24" t="str">
+      <c r="C22" s="91"/>
+      <c r="D22" s="92"/>
+      <c r="E22" s="34"/>
+      <c r="F22" s="93"/>
+      <c r="G22" s="34"/>
+      <c r="H22" s="94" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="I22" s="25" t="str">
+      <c r="I22" s="95" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -3456,7 +3227,7 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K22" s="24" t="str">
+      <c r="K22" s="94" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -3464,7 +3235,7 @@
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="M22" s="24" t="str">
+      <c r="M22" s="94" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -3472,42 +3243,42 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="O22" s="33" t="str">
+      <c r="O22" s="96" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="P22" s="48"/>
-      <c r="Q22" s="57" t="str">
+      <c r="P22" s="91"/>
+      <c r="Q22" s="97" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="R22" s="49"/>
-      <c r="S22" s="57" t="str">
+      <c r="R22" s="34"/>
+      <c r="S22" s="97" t="str">
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="T22" s="50"/>
-      <c r="U22" s="24" t="str">
+      <c r="T22" s="34"/>
+      <c r="U22" s="94" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="V22" s="25" t="str">
+      <c r="V22" s="95" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="W22" s="35" t="str">
+      <c r="W22" s="98" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="X22" s="60"/>
-      <c r="Y22" s="116"/>
-      <c r="Z22" s="117"/>
-      <c r="AA22" s="117"/>
-      <c r="AB22" s="117"/>
-      <c r="AC22" s="117"/>
-      <c r="AD22" s="118"/>
-      <c r="AE22" s="71"/>
-      <c r="AF22" s="1" t="str">
+      <c r="X22" s="35"/>
+      <c r="Y22" s="50"/>
+      <c r="Z22" s="51"/>
+      <c r="AA22" s="51"/>
+      <c r="AB22" s="51"/>
+      <c r="AC22" s="51"/>
+      <c r="AD22" s="52"/>
+      <c r="AE22" s="45"/>
+      <c r="AF22" s="3" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
@@ -3521,16 +3292,16 @@
         <f t="shared" si="12"/>
         <v>46158</v>
       </c>
-      <c r="C23" s="48"/>
-      <c r="D23" s="45"/>
-      <c r="E23" s="49"/>
-      <c r="F23" s="46"/>
-      <c r="G23" s="50"/>
-      <c r="H23" s="24" t="str">
+      <c r="C23" s="91"/>
+      <c r="D23" s="92"/>
+      <c r="E23" s="34"/>
+      <c r="F23" s="93"/>
+      <c r="G23" s="34"/>
+      <c r="H23" s="94" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="I23" s="25" t="str">
+      <c r="I23" s="95" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -3538,7 +3309,7 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K23" s="24" t="str">
+      <c r="K23" s="94" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -3546,7 +3317,7 @@
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="M23" s="24" t="str">
+      <c r="M23" s="94" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -3554,42 +3325,42 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="O23" s="33" t="str">
+      <c r="O23" s="96" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="P23" s="48"/>
-      <c r="Q23" s="57" t="str">
+      <c r="P23" s="91"/>
+      <c r="Q23" s="97" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="R23" s="49"/>
-      <c r="S23" s="57" t="str">
+      <c r="R23" s="34"/>
+      <c r="S23" s="97" t="str">
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="T23" s="50"/>
-      <c r="U23" s="24" t="str">
+      <c r="T23" s="34"/>
+      <c r="U23" s="94" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="V23" s="25" t="str">
+      <c r="V23" s="95" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="W23" s="35" t="str">
+      <c r="W23" s="98" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="X23" s="60"/>
-      <c r="Y23" s="116"/>
-      <c r="Z23" s="117"/>
-      <c r="AA23" s="117"/>
-      <c r="AB23" s="117"/>
-      <c r="AC23" s="117"/>
-      <c r="AD23" s="118"/>
-      <c r="AE23" s="71"/>
-      <c r="AF23" s="1" t="str">
+      <c r="X23" s="35"/>
+      <c r="Y23" s="50"/>
+      <c r="Z23" s="51"/>
+      <c r="AA23" s="51"/>
+      <c r="AB23" s="51"/>
+      <c r="AC23" s="51"/>
+      <c r="AD23" s="52"/>
+      <c r="AE23" s="45"/>
+      <c r="AF23" s="3" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
@@ -3603,16 +3374,16 @@
         <f t="shared" si="12"/>
         <v>46159</v>
       </c>
-      <c r="C24" s="48"/>
-      <c r="D24" s="45"/>
-      <c r="E24" s="49"/>
-      <c r="F24" s="46"/>
-      <c r="G24" s="50"/>
-      <c r="H24" s="24" t="str">
+      <c r="C24" s="91"/>
+      <c r="D24" s="92"/>
+      <c r="E24" s="34"/>
+      <c r="F24" s="93"/>
+      <c r="G24" s="34"/>
+      <c r="H24" s="94" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="I24" s="25" t="str">
+      <c r="I24" s="95" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -3620,7 +3391,7 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K24" s="24" t="str">
+      <c r="K24" s="94" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -3628,7 +3399,7 @@
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="M24" s="24" t="str">
+      <c r="M24" s="94" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -3636,42 +3407,42 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="O24" s="33" t="str">
+      <c r="O24" s="96" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="P24" s="48"/>
-      <c r="Q24" s="57" t="str">
+      <c r="P24" s="91"/>
+      <c r="Q24" s="97" t="str">
         <f>IF(P24="","",P24/"01:00:00")</f>
         <v/>
       </c>
-      <c r="R24" s="49"/>
-      <c r="S24" s="57" t="str">
+      <c r="R24" s="34"/>
+      <c r="S24" s="97" t="str">
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="T24" s="50"/>
-      <c r="U24" s="24" t="str">
+      <c r="T24" s="34"/>
+      <c r="U24" s="94" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="V24" s="25" t="str">
+      <c r="V24" s="95" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="W24" s="35" t="str">
+      <c r="W24" s="98" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="X24" s="60"/>
-      <c r="Y24" s="116"/>
-      <c r="Z24" s="117"/>
-      <c r="AA24" s="117"/>
-      <c r="AB24" s="117"/>
-      <c r="AC24" s="117"/>
-      <c r="AD24" s="118"/>
-      <c r="AE24" s="71"/>
-      <c r="AF24" s="1" t="str">
+      <c r="X24" s="35"/>
+      <c r="Y24" s="50"/>
+      <c r="Z24" s="51"/>
+      <c r="AA24" s="51"/>
+      <c r="AB24" s="51"/>
+      <c r="AC24" s="51"/>
+      <c r="AD24" s="52"/>
+      <c r="AE24" s="45"/>
+      <c r="AF24" s="3" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
@@ -3685,16 +3456,16 @@
         <f t="shared" si="12"/>
         <v>46160</v>
       </c>
-      <c r="C25" s="48"/>
-      <c r="D25" s="45"/>
-      <c r="E25" s="49"/>
-      <c r="F25" s="46"/>
-      <c r="G25" s="50"/>
-      <c r="H25" s="24" t="str">
+      <c r="C25" s="91"/>
+      <c r="D25" s="92"/>
+      <c r="E25" s="34"/>
+      <c r="F25" s="93"/>
+      <c r="G25" s="34"/>
+      <c r="H25" s="94" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="I25" s="25" t="str">
+      <c r="I25" s="95" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -3702,7 +3473,7 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K25" s="24" t="str">
+      <c r="K25" s="94" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -3710,7 +3481,7 @@
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="M25" s="24" t="str">
+      <c r="M25" s="94" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -3718,42 +3489,42 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="O25" s="33" t="str">
+      <c r="O25" s="96" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="P25" s="48"/>
-      <c r="Q25" s="57" t="str">
+      <c r="P25" s="91"/>
+      <c r="Q25" s="97" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="R25" s="49"/>
-      <c r="S25" s="57" t="str">
+      <c r="R25" s="34"/>
+      <c r="S25" s="97" t="str">
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="T25" s="50"/>
-      <c r="U25" s="24" t="str">
+      <c r="T25" s="34"/>
+      <c r="U25" s="94" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="V25" s="25" t="str">
+      <c r="V25" s="95" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="W25" s="35" t="str">
+      <c r="W25" s="98" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="X25" s="60"/>
-      <c r="Y25" s="116"/>
-      <c r="Z25" s="117"/>
-      <c r="AA25" s="117"/>
-      <c r="AB25" s="117"/>
-      <c r="AC25" s="117"/>
-      <c r="AD25" s="118"/>
-      <c r="AE25" s="71"/>
-      <c r="AF25" s="1" t="str">
+      <c r="X25" s="35"/>
+      <c r="Y25" s="50"/>
+      <c r="Z25" s="51"/>
+      <c r="AA25" s="51"/>
+      <c r="AB25" s="51"/>
+      <c r="AC25" s="51"/>
+      <c r="AD25" s="52"/>
+      <c r="AE25" s="45"/>
+      <c r="AF25" s="3" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
@@ -3767,16 +3538,16 @@
         <f>A26</f>
         <v>46161</v>
       </c>
-      <c r="C26" s="48"/>
-      <c r="D26" s="45"/>
-      <c r="E26" s="49"/>
-      <c r="F26" s="46"/>
-      <c r="G26" s="50"/>
-      <c r="H26" s="24" t="str">
+      <c r="C26" s="91"/>
+      <c r="D26" s="92"/>
+      <c r="E26" s="34"/>
+      <c r="F26" s="93"/>
+      <c r="G26" s="34"/>
+      <c r="H26" s="94" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="I26" s="25" t="str">
+      <c r="I26" s="95" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -3784,7 +3555,7 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K26" s="24" t="str">
+      <c r="K26" s="94" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -3792,7 +3563,7 @@
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="M26" s="24" t="str">
+      <c r="M26" s="94" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -3800,48 +3571,48 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="O26" s="33" t="str">
+      <c r="O26" s="96" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="P26" s="48"/>
-      <c r="Q26" s="57" t="str">
+      <c r="P26" s="91"/>
+      <c r="Q26" s="97" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="R26" s="49"/>
-      <c r="S26" s="57" t="str">
+      <c r="R26" s="34"/>
+      <c r="S26" s="97" t="str">
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="T26" s="50"/>
-      <c r="U26" s="24" t="str">
+      <c r="T26" s="34"/>
+      <c r="U26" s="94" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="V26" s="25" t="str">
+      <c r="V26" s="95" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="W26" s="35" t="str">
+      <c r="W26" s="98" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="X26" s="60"/>
-      <c r="Y26" s="116"/>
-      <c r="Z26" s="117"/>
-      <c r="AA26" s="117"/>
-      <c r="AB26" s="117"/>
-      <c r="AC26" s="117"/>
-      <c r="AD26" s="118"/>
-      <c r="AE26" s="71"/>
-      <c r="AF26" s="1" t="str">
+      <c r="X26" s="35"/>
+      <c r="Y26" s="50"/>
+      <c r="Z26" s="51"/>
+      <c r="AA26" s="51"/>
+      <c r="AB26" s="51"/>
+      <c r="AC26" s="51"/>
+      <c r="AD26" s="52"/>
+      <c r="AE26" s="45"/>
+      <c r="AF26" s="3" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
     </row>
     <row r="27" spans="1:32" ht="18" customHeight="1">
-      <c r="A27" s="75">
+      <c r="A27" s="49">
         <f t="shared" si="16"/>
         <v>46162</v>
       </c>
@@ -3849,16 +3620,16 @@
         <f t="shared" si="12"/>
         <v>46162</v>
       </c>
-      <c r="C27" s="48"/>
-      <c r="D27" s="45"/>
-      <c r="E27" s="49"/>
-      <c r="F27" s="46"/>
-      <c r="G27" s="50"/>
-      <c r="H27" s="24" t="str">
+      <c r="C27" s="91"/>
+      <c r="D27" s="92"/>
+      <c r="E27" s="34"/>
+      <c r="F27" s="93"/>
+      <c r="G27" s="34"/>
+      <c r="H27" s="94" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="I27" s="25" t="str">
+      <c r="I27" s="95" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -3866,7 +3637,7 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K27" s="24" t="str">
+      <c r="K27" s="94" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -3874,7 +3645,7 @@
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="M27" s="24" t="str">
+      <c r="M27" s="94" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -3882,48 +3653,48 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="O27" s="33" t="str">
+      <c r="O27" s="96" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="P27" s="48"/>
-      <c r="Q27" s="57" t="str">
+      <c r="P27" s="91"/>
+      <c r="Q27" s="97" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="R27" s="49"/>
-      <c r="S27" s="57" t="str">
+      <c r="R27" s="34"/>
+      <c r="S27" s="97" t="str">
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="T27" s="50"/>
-      <c r="U27" s="24" t="str">
+      <c r="T27" s="34"/>
+      <c r="U27" s="94" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="V27" s="25" t="str">
+      <c r="V27" s="95" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="W27" s="35" t="str">
+      <c r="W27" s="98" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="X27" s="60"/>
-      <c r="Y27" s="116"/>
-      <c r="Z27" s="117"/>
-      <c r="AA27" s="117"/>
-      <c r="AB27" s="117"/>
-      <c r="AC27" s="117"/>
-      <c r="AD27" s="118"/>
-      <c r="AE27" s="71"/>
-      <c r="AF27" s="1" t="str">
+      <c r="X27" s="35"/>
+      <c r="Y27" s="50"/>
+      <c r="Z27" s="51"/>
+      <c r="AA27" s="51"/>
+      <c r="AB27" s="51"/>
+      <c r="AC27" s="51"/>
+      <c r="AD27" s="52"/>
+      <c r="AE27" s="45"/>
+      <c r="AF27" s="3" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
     </row>
     <row r="28" spans="1:32" ht="18" customHeight="1" thickBot="1">
-      <c r="A28" s="75">
+      <c r="A28" s="49">
         <f t="shared" si="16"/>
         <v>46163</v>
       </c>
@@ -3931,16 +3702,16 @@
         <f t="shared" si="12"/>
         <v>46163</v>
       </c>
-      <c r="C28" s="48"/>
-      <c r="D28" s="45"/>
-      <c r="E28" s="49"/>
-      <c r="F28" s="46"/>
-      <c r="G28" s="50"/>
-      <c r="H28" s="24" t="str">
+      <c r="C28" s="91"/>
+      <c r="D28" s="92"/>
+      <c r="E28" s="34"/>
+      <c r="F28" s="93"/>
+      <c r="G28" s="34"/>
+      <c r="H28" s="94" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="I28" s="25" t="str">
+      <c r="I28" s="95" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -3948,7 +3719,7 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K28" s="24" t="str">
+      <c r="K28" s="94" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -3956,7 +3727,7 @@
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="M28" s="24" t="str">
+      <c r="M28" s="94" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -3964,42 +3735,42 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="O28" s="33" t="str">
+      <c r="O28" s="96" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="P28" s="48"/>
-      <c r="Q28" s="57" t="str">
+      <c r="P28" s="91"/>
+      <c r="Q28" s="97" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="R28" s="49"/>
-      <c r="S28" s="57" t="str">
+      <c r="R28" s="34"/>
+      <c r="S28" s="97" t="str">
         <f>IF(R28="","",R28/"01:00:00")</f>
         <v/>
       </c>
-      <c r="T28" s="50"/>
-      <c r="U28" s="24" t="str">
+      <c r="T28" s="34"/>
+      <c r="U28" s="94" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="V28" s="25" t="str">
+      <c r="V28" s="95" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="W28" s="35" t="str">
+      <c r="W28" s="98" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="X28" s="60"/>
-      <c r="Y28" s="122"/>
-      <c r="Z28" s="120"/>
-      <c r="AA28" s="120"/>
-      <c r="AB28" s="120"/>
-      <c r="AC28" s="120"/>
-      <c r="AD28" s="121"/>
-      <c r="AE28" s="71"/>
-      <c r="AF28" s="1" t="str">
+      <c r="X28" s="35"/>
+      <c r="Y28" s="56"/>
+      <c r="Z28" s="57"/>
+      <c r="AA28" s="57"/>
+      <c r="AB28" s="57"/>
+      <c r="AC28" s="57"/>
+      <c r="AD28" s="58"/>
+      <c r="AE28" s="45"/>
+      <c r="AF28" s="3" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
@@ -4013,16 +3784,16 @@
         <f t="shared" si="12"/>
         <v>46164</v>
       </c>
-      <c r="C29" s="48"/>
-      <c r="D29" s="45"/>
-      <c r="E29" s="49"/>
-      <c r="F29" s="46"/>
-      <c r="G29" s="50"/>
-      <c r="H29" s="24" t="str">
+      <c r="C29" s="91"/>
+      <c r="D29" s="92"/>
+      <c r="E29" s="34"/>
+      <c r="F29" s="93"/>
+      <c r="G29" s="34"/>
+      <c r="H29" s="94" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="I29" s="25" t="str">
+      <c r="I29" s="95" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -4030,7 +3801,7 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K29" s="24" t="str">
+      <c r="K29" s="94" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -4038,7 +3809,7 @@
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="M29" s="24" t="str">
+      <c r="M29" s="94" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -4046,36 +3817,36 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="O29" s="33" t="str">
+      <c r="O29" s="96" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="P29" s="48"/>
-      <c r="Q29" s="57"/>
-      <c r="R29" s="49"/>
-      <c r="S29" s="57"/>
-      <c r="T29" s="50"/>
-      <c r="U29" s="24" t="str">
+      <c r="P29" s="91"/>
+      <c r="Q29" s="97"/>
+      <c r="R29" s="34"/>
+      <c r="S29" s="97"/>
+      <c r="T29" s="34"/>
+      <c r="U29" s="94" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="V29" s="25" t="str">
+      <c r="V29" s="95" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="W29" s="35" t="str">
+      <c r="W29" s="98" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="X29" s="60"/>
-      <c r="Y29" s="116"/>
-      <c r="Z29" s="117"/>
-      <c r="AA29" s="117"/>
-      <c r="AB29" s="117"/>
-      <c r="AC29" s="117"/>
-      <c r="AD29" s="118"/>
-      <c r="AE29" s="71"/>
-      <c r="AF29" s="1" t="str">
+      <c r="X29" s="35"/>
+      <c r="Y29" s="50"/>
+      <c r="Z29" s="51"/>
+      <c r="AA29" s="51"/>
+      <c r="AB29" s="51"/>
+      <c r="AC29" s="51"/>
+      <c r="AD29" s="52"/>
+      <c r="AE29" s="45"/>
+      <c r="AF29" s="3" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
@@ -4089,16 +3860,16 @@
         <f t="shared" si="12"/>
         <v>46165</v>
       </c>
-      <c r="C30" s="48"/>
-      <c r="D30" s="45"/>
-      <c r="E30" s="49"/>
-      <c r="F30" s="46"/>
-      <c r="G30" s="50"/>
-      <c r="H30" s="24" t="str">
+      <c r="C30" s="91"/>
+      <c r="D30" s="92"/>
+      <c r="E30" s="34"/>
+      <c r="F30" s="93"/>
+      <c r="G30" s="34"/>
+      <c r="H30" s="94" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="I30" s="25" t="str">
+      <c r="I30" s="95" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -4106,7 +3877,7 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K30" s="24" t="str">
+      <c r="K30" s="94" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -4114,7 +3885,7 @@
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="M30" s="24" t="str">
+      <c r="M30" s="94" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -4122,36 +3893,36 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="O30" s="33" t="str">
+      <c r="O30" s="96" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="P30" s="48"/>
-      <c r="Q30" s="57"/>
-      <c r="R30" s="49"/>
-      <c r="S30" s="57"/>
-      <c r="T30" s="50"/>
-      <c r="U30" s="24" t="str">
+      <c r="P30" s="91"/>
+      <c r="Q30" s="97"/>
+      <c r="R30" s="34"/>
+      <c r="S30" s="97"/>
+      <c r="T30" s="34"/>
+      <c r="U30" s="94" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="V30" s="25" t="str">
+      <c r="V30" s="95" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="W30" s="35" t="str">
+      <c r="W30" s="98" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="X30" s="60"/>
-      <c r="Y30" s="116"/>
-      <c r="Z30" s="117"/>
-      <c r="AA30" s="117"/>
-      <c r="AB30" s="117"/>
-      <c r="AC30" s="117"/>
-      <c r="AD30" s="118"/>
-      <c r="AE30" s="71"/>
-      <c r="AF30" s="1" t="str">
+      <c r="X30" s="35"/>
+      <c r="Y30" s="50"/>
+      <c r="Z30" s="51"/>
+      <c r="AA30" s="51"/>
+      <c r="AB30" s="51"/>
+      <c r="AC30" s="51"/>
+      <c r="AD30" s="52"/>
+      <c r="AE30" s="45"/>
+      <c r="AF30" s="3" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
@@ -4165,16 +3936,16 @@
         <f t="shared" si="12"/>
         <v>46166</v>
       </c>
-      <c r="C31" s="48"/>
-      <c r="D31" s="45"/>
-      <c r="E31" s="49"/>
-      <c r="F31" s="46"/>
-      <c r="G31" s="50"/>
-      <c r="H31" s="24" t="str">
+      <c r="C31" s="91"/>
+      <c r="D31" s="92"/>
+      <c r="E31" s="34"/>
+      <c r="F31" s="93"/>
+      <c r="G31" s="34"/>
+      <c r="H31" s="94" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="I31" s="25" t="str">
+      <c r="I31" s="95" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -4182,7 +3953,7 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K31" s="24" t="str">
+      <c r="K31" s="94" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -4190,7 +3961,7 @@
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="M31" s="24" t="str">
+      <c r="M31" s="94" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -4198,36 +3969,36 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="O31" s="33" t="str">
+      <c r="O31" s="96" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="P31" s="48"/>
-      <c r="Q31" s="57"/>
-      <c r="R31" s="49"/>
-      <c r="S31" s="57"/>
-      <c r="T31" s="50"/>
-      <c r="U31" s="24" t="str">
+      <c r="P31" s="91"/>
+      <c r="Q31" s="97"/>
+      <c r="R31" s="34"/>
+      <c r="S31" s="97"/>
+      <c r="T31" s="34"/>
+      <c r="U31" s="94" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="V31" s="25" t="str">
+      <c r="V31" s="95" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="W31" s="35" t="str">
+      <c r="W31" s="98" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="X31" s="60"/>
-      <c r="Y31" s="116"/>
-      <c r="Z31" s="117"/>
-      <c r="AA31" s="117"/>
-      <c r="AB31" s="117"/>
-      <c r="AC31" s="117"/>
-      <c r="AD31" s="118"/>
-      <c r="AE31" s="71"/>
-      <c r="AF31" s="1" t="str">
+      <c r="X31" s="35"/>
+      <c r="Y31" s="50"/>
+      <c r="Z31" s="51"/>
+      <c r="AA31" s="51"/>
+      <c r="AB31" s="51"/>
+      <c r="AC31" s="51"/>
+      <c r="AD31" s="52"/>
+      <c r="AE31" s="45"/>
+      <c r="AF31" s="3" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
@@ -4241,16 +4012,16 @@
         <f t="shared" si="12"/>
         <v>46167</v>
       </c>
-      <c r="C32" s="48"/>
-      <c r="D32" s="45"/>
-      <c r="E32" s="49"/>
-      <c r="F32" s="46"/>
-      <c r="G32" s="50"/>
-      <c r="H32" s="24" t="str">
+      <c r="C32" s="91"/>
+      <c r="D32" s="92"/>
+      <c r="E32" s="34"/>
+      <c r="F32" s="93"/>
+      <c r="G32" s="34"/>
+      <c r="H32" s="94" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="I32" s="25" t="str">
+      <c r="I32" s="95" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -4258,7 +4029,7 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K32" s="24" t="str">
+      <c r="K32" s="94" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -4266,7 +4037,7 @@
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="M32" s="24" t="str">
+      <c r="M32" s="94" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -4274,36 +4045,36 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="O32" s="33" t="str">
+      <c r="O32" s="96" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="P32" s="48"/>
-      <c r="Q32" s="57"/>
-      <c r="R32" s="49"/>
-      <c r="S32" s="57"/>
-      <c r="T32" s="50"/>
-      <c r="U32" s="24" t="str">
+      <c r="P32" s="91"/>
+      <c r="Q32" s="97"/>
+      <c r="R32" s="34"/>
+      <c r="S32" s="97"/>
+      <c r="T32" s="34"/>
+      <c r="U32" s="94" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="V32" s="25" t="str">
+      <c r="V32" s="95" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="W32" s="35" t="str">
+      <c r="W32" s="98" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="X32" s="60"/>
-      <c r="Y32" s="116"/>
-      <c r="Z32" s="117"/>
-      <c r="AA32" s="117"/>
-      <c r="AB32" s="117"/>
-      <c r="AC32" s="117"/>
-      <c r="AD32" s="118"/>
-      <c r="AE32" s="71"/>
-      <c r="AF32" s="1" t="str">
+      <c r="X32" s="35"/>
+      <c r="Y32" s="50"/>
+      <c r="Z32" s="51"/>
+      <c r="AA32" s="51"/>
+      <c r="AB32" s="51"/>
+      <c r="AC32" s="51"/>
+      <c r="AD32" s="52"/>
+      <c r="AE32" s="45"/>
+      <c r="AF32" s="3" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
@@ -4317,16 +4088,16 @@
         <f t="shared" si="12"/>
         <v>46168</v>
       </c>
-      <c r="C33" s="48"/>
-      <c r="D33" s="45"/>
-      <c r="E33" s="49"/>
-      <c r="F33" s="46"/>
-      <c r="G33" s="50"/>
-      <c r="H33" s="24" t="str">
+      <c r="C33" s="91"/>
+      <c r="D33" s="92"/>
+      <c r="E33" s="34"/>
+      <c r="F33" s="93"/>
+      <c r="G33" s="34"/>
+      <c r="H33" s="94" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="I33" s="25" t="str">
+      <c r="I33" s="95" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -4334,7 +4105,7 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K33" s="24" t="str">
+      <c r="K33" s="94" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -4342,7 +4113,7 @@
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="M33" s="24" t="str">
+      <c r="M33" s="94" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -4350,36 +4121,36 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="O33" s="33" t="str">
+      <c r="O33" s="96" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="P33" s="48"/>
-      <c r="Q33" s="57"/>
-      <c r="R33" s="49"/>
-      <c r="S33" s="57"/>
-      <c r="T33" s="50"/>
-      <c r="U33" s="24" t="str">
+      <c r="P33" s="91"/>
+      <c r="Q33" s="97"/>
+      <c r="R33" s="34"/>
+      <c r="S33" s="97"/>
+      <c r="T33" s="34"/>
+      <c r="U33" s="94" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="V33" s="25" t="str">
+      <c r="V33" s="95" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="W33" s="35" t="str">
+      <c r="W33" s="98" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="X33" s="60"/>
-      <c r="Y33" s="116"/>
-      <c r="Z33" s="117"/>
-      <c r="AA33" s="117"/>
-      <c r="AB33" s="117"/>
-      <c r="AC33" s="117"/>
-      <c r="AD33" s="118"/>
-      <c r="AE33" s="71"/>
-      <c r="AF33" s="1" t="str">
+      <c r="X33" s="35"/>
+      <c r="Y33" s="50"/>
+      <c r="Z33" s="51"/>
+      <c r="AA33" s="51"/>
+      <c r="AB33" s="51"/>
+      <c r="AC33" s="51"/>
+      <c r="AD33" s="52"/>
+      <c r="AE33" s="45"/>
+      <c r="AF33" s="3" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
@@ -4393,16 +4164,16 @@
         <f t="shared" si="12"/>
         <v>46169</v>
       </c>
-      <c r="C34" s="48"/>
-      <c r="D34" s="45"/>
-      <c r="E34" s="49"/>
-      <c r="F34" s="46"/>
-      <c r="G34" s="50"/>
-      <c r="H34" s="24" t="str">
+      <c r="C34" s="91"/>
+      <c r="D34" s="92"/>
+      <c r="E34" s="34"/>
+      <c r="F34" s="93"/>
+      <c r="G34" s="34"/>
+      <c r="H34" s="94" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="I34" s="25" t="str">
+      <c r="I34" s="95" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -4410,7 +4181,7 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K34" s="24" t="str">
+      <c r="K34" s="94" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -4418,7 +4189,7 @@
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="M34" s="24" t="str">
+      <c r="M34" s="94" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -4426,36 +4197,36 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="O34" s="33" t="str">
+      <c r="O34" s="96" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="P34" s="48"/>
-      <c r="Q34" s="57"/>
-      <c r="R34" s="49"/>
-      <c r="S34" s="57"/>
-      <c r="T34" s="50"/>
-      <c r="U34" s="24" t="str">
+      <c r="P34" s="91"/>
+      <c r="Q34" s="97"/>
+      <c r="R34" s="34"/>
+      <c r="S34" s="97"/>
+      <c r="T34" s="34"/>
+      <c r="U34" s="94" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="V34" s="25" t="str">
+      <c r="V34" s="95" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="W34" s="35" t="str">
+      <c r="W34" s="98" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="X34" s="60"/>
-      <c r="Y34" s="116"/>
-      <c r="Z34" s="117"/>
-      <c r="AA34" s="117"/>
-      <c r="AB34" s="117"/>
-      <c r="AC34" s="117"/>
-      <c r="AD34" s="118"/>
-      <c r="AE34" s="71"/>
-      <c r="AF34" s="1" t="str">
+      <c r="X34" s="35"/>
+      <c r="Y34" s="50"/>
+      <c r="Z34" s="51"/>
+      <c r="AA34" s="51"/>
+      <c r="AB34" s="51"/>
+      <c r="AC34" s="51"/>
+      <c r="AD34" s="52"/>
+      <c r="AE34" s="45"/>
+      <c r="AF34" s="3" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
@@ -4469,16 +4240,16 @@
         <f t="shared" si="12"/>
         <v>46170</v>
       </c>
-      <c r="C35" s="48"/>
-      <c r="D35" s="45"/>
-      <c r="E35" s="49"/>
-      <c r="F35" s="46"/>
-      <c r="G35" s="50"/>
-      <c r="H35" s="24" t="str">
+      <c r="C35" s="91"/>
+      <c r="D35" s="92"/>
+      <c r="E35" s="34"/>
+      <c r="F35" s="93"/>
+      <c r="G35" s="34"/>
+      <c r="H35" s="94" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="I35" s="25" t="str">
+      <c r="I35" s="95" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -4486,7 +4257,7 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K35" s="24" t="str">
+      <c r="K35" s="94" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -4494,7 +4265,7 @@
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="M35" s="24" t="str">
+      <c r="M35" s="94" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -4502,36 +4273,36 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="O35" s="33" t="str">
+      <c r="O35" s="96" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="P35" s="48"/>
-      <c r="Q35" s="57"/>
-      <c r="R35" s="49"/>
-      <c r="S35" s="57"/>
-      <c r="T35" s="50"/>
-      <c r="U35" s="24" t="str">
+      <c r="P35" s="91"/>
+      <c r="Q35" s="97"/>
+      <c r="R35" s="34"/>
+      <c r="S35" s="97"/>
+      <c r="T35" s="34"/>
+      <c r="U35" s="94" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="V35" s="25" t="str">
+      <c r="V35" s="95" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="W35" s="35" t="str">
+      <c r="W35" s="98" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="X35" s="60"/>
-      <c r="Y35" s="116"/>
-      <c r="Z35" s="117"/>
-      <c r="AA35" s="117"/>
-      <c r="AB35" s="117"/>
-      <c r="AC35" s="117"/>
-      <c r="AD35" s="118"/>
-      <c r="AE35" s="71"/>
-      <c r="AF35" s="1" t="str">
+      <c r="X35" s="35"/>
+      <c r="Y35" s="50"/>
+      <c r="Z35" s="51"/>
+      <c r="AA35" s="51"/>
+      <c r="AB35" s="51"/>
+      <c r="AC35" s="51"/>
+      <c r="AD35" s="52"/>
+      <c r="AE35" s="45"/>
+      <c r="AF35" s="3" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
@@ -4545,16 +4316,16 @@
         <f t="shared" ca="1" si="12"/>
         <v>46171</v>
       </c>
-      <c r="C36" s="48"/>
-      <c r="D36" s="45"/>
-      <c r="E36" s="49"/>
-      <c r="F36" s="46"/>
-      <c r="G36" s="50"/>
-      <c r="H36" s="24" t="str">
+      <c r="C36" s="91"/>
+      <c r="D36" s="92"/>
+      <c r="E36" s="34"/>
+      <c r="F36" s="93"/>
+      <c r="G36" s="34"/>
+      <c r="H36" s="94" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="I36" s="25" t="str">
+      <c r="I36" s="95" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -4562,7 +4333,7 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K36" s="24" t="str">
+      <c r="K36" s="94" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -4570,7 +4341,7 @@
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="M36" s="24" t="str">
+      <c r="M36" s="94" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -4578,36 +4349,36 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="O36" s="33" t="str">
+      <c r="O36" s="96" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="P36" s="48"/>
-      <c r="Q36" s="57"/>
-      <c r="R36" s="49"/>
-      <c r="S36" s="57"/>
-      <c r="T36" s="50"/>
-      <c r="U36" s="24" t="str">
+      <c r="P36" s="91"/>
+      <c r="Q36" s="97"/>
+      <c r="R36" s="34"/>
+      <c r="S36" s="97"/>
+      <c r="T36" s="34"/>
+      <c r="U36" s="94" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="V36" s="25" t="str">
+      <c r="V36" s="95" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="W36" s="35" t="str">
+      <c r="W36" s="98" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="X36" s="60"/>
-      <c r="Y36" s="116"/>
-      <c r="Z36" s="117"/>
-      <c r="AA36" s="117"/>
-      <c r="AB36" s="117"/>
-      <c r="AC36" s="117"/>
-      <c r="AD36" s="118"/>
-      <c r="AE36" s="71"/>
-      <c r="AF36" s="1" t="str">
+      <c r="X36" s="35"/>
+      <c r="Y36" s="50"/>
+      <c r="Z36" s="51"/>
+      <c r="AA36" s="51"/>
+      <c r="AB36" s="51"/>
+      <c r="AC36" s="51"/>
+      <c r="AD36" s="52"/>
+      <c r="AE36" s="45"/>
+      <c r="AF36" s="3" t="str">
         <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
@@ -4621,16 +4392,16 @@
         <f t="shared" ca="1" si="12"/>
         <v>46172</v>
       </c>
-      <c r="C37" s="48"/>
-      <c r="D37" s="45"/>
-      <c r="E37" s="49"/>
-      <c r="F37" s="46"/>
-      <c r="G37" s="50"/>
-      <c r="H37" s="24" t="str">
+      <c r="C37" s="91"/>
+      <c r="D37" s="92"/>
+      <c r="E37" s="34"/>
+      <c r="F37" s="93"/>
+      <c r="G37" s="34"/>
+      <c r="H37" s="94" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="I37" s="25" t="str">
+      <c r="I37" s="95" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -4638,7 +4409,7 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K37" s="24" t="str">
+      <c r="K37" s="94" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -4646,7 +4417,7 @@
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="M37" s="24" t="str">
+      <c r="M37" s="94" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -4654,42 +4425,42 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="O37" s="33" t="str">
+      <c r="O37" s="96" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="P37" s="48"/>
-      <c r="Q37" s="57" t="str">
+      <c r="P37" s="91"/>
+      <c r="Q37" s="97" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="R37" s="49"/>
-      <c r="S37" s="57" t="str">
+      <c r="R37" s="34"/>
+      <c r="S37" s="97" t="str">
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="T37" s="50"/>
-      <c r="U37" s="24" t="str">
+      <c r="T37" s="34"/>
+      <c r="U37" s="94" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="V37" s="25" t="str">
+      <c r="V37" s="95" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="W37" s="35" t="str">
+      <c r="W37" s="98" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="X37" s="60"/>
-      <c r="Y37" s="116"/>
-      <c r="Z37" s="117"/>
-      <c r="AA37" s="117"/>
-      <c r="AB37" s="117"/>
-      <c r="AC37" s="117"/>
-      <c r="AD37" s="118"/>
-      <c r="AE37" s="71"/>
-      <c r="AF37" s="1" t="str">
+      <c r="X37" s="35"/>
+      <c r="Y37" s="50"/>
+      <c r="Z37" s="51"/>
+      <c r="AA37" s="51"/>
+      <c r="AB37" s="51"/>
+      <c r="AC37" s="51"/>
+      <c r="AD37" s="52"/>
+      <c r="AE37" s="45"/>
+      <c r="AF37" s="3" t="str">
         <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
@@ -4703,30 +4474,30 @@
         <f t="shared" ca="1" si="12"/>
         <v>46173</v>
       </c>
-      <c r="C38" s="51"/>
-      <c r="D38" s="45" t="str">
+      <c r="C38" s="91"/>
+      <c r="D38" s="92" t="str">
         <f>IF(C38="","",C38/"01:00:00")</f>
         <v/>
       </c>
-      <c r="E38" s="52"/>
-      <c r="F38" s="46" t="str">
+      <c r="E38" s="34"/>
+      <c r="F38" s="93" t="str">
         <f>IF(E38="","",E38/"01:00:00")</f>
         <v/>
       </c>
-      <c r="G38" s="53"/>
-      <c r="H38" s="26" t="str">
+      <c r="G38" s="34"/>
+      <c r="H38" s="94" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="I38" s="27" t="str">
+      <c r="I38" s="95" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J38" s="18" t="str">
+      <c r="J38" s="8" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K38" s="24" t="str">
+      <c r="K38" s="94" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -4734,7 +4505,7 @@
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="M38" s="24" t="str">
+      <c r="M38" s="94" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -4742,104 +4513,104 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="O38" s="33" t="str">
+      <c r="O38" s="96" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="P38" s="51"/>
-      <c r="Q38" s="58" t="str">
+      <c r="P38" s="91"/>
+      <c r="Q38" s="97" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="R38" s="52"/>
-      <c r="S38" s="58" t="str">
+      <c r="R38" s="34"/>
+      <c r="S38" s="97" t="str">
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="T38" s="53"/>
-      <c r="U38" s="26" t="str">
+      <c r="T38" s="34"/>
+      <c r="U38" s="94" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="V38" s="27" t="str">
+      <c r="V38" s="95" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="W38" s="36" t="str">
+      <c r="W38" s="98" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="X38" s="61"/>
-      <c r="Y38" s="123"/>
-      <c r="Z38" s="124"/>
-      <c r="AA38" s="124"/>
-      <c r="AB38" s="124"/>
-      <c r="AC38" s="124"/>
-      <c r="AD38" s="125"/>
-      <c r="AE38" s="72"/>
-      <c r="AF38" s="1" t="str">
+      <c r="X38" s="35"/>
+      <c r="Y38" s="53"/>
+      <c r="Z38" s="54"/>
+      <c r="AA38" s="54"/>
+      <c r="AB38" s="54"/>
+      <c r="AC38" s="54"/>
+      <c r="AD38" s="55"/>
+      <c r="AE38" s="46"/>
+      <c r="AF38" s="3" t="str">
         <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
     </row>
     <row r="39" spans="1:32" ht="22.5" customHeight="1" thickBot="1">
-      <c r="A39" s="85" t="s">
+      <c r="A39" s="65" t="s">
         <v>9</v>
       </c>
-      <c r="B39" s="86"/>
-      <c r="C39" s="31">
+      <c r="B39" s="79"/>
+      <c r="C39" s="24">
         <f ca="1">COUNTIF(AF8:AF38,"稼働日")</f>
         <v>0</v>
       </c>
-      <c r="D39" s="31"/>
-      <c r="E39" s="41" t="s">
+      <c r="D39" s="24"/>
+      <c r="E39" s="30" t="s">
         <v>10</v>
       </c>
       <c r="F39" s="10"/>
-      <c r="G39" s="28" t="s">
+      <c r="G39" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="H39" s="21"/>
-      <c r="I39" s="21"/>
-      <c r="J39" s="29"/>
-      <c r="K39" s="29">
+      <c r="H39" s="20"/>
+      <c r="I39" s="20"/>
+      <c r="J39" s="22"/>
+      <c r="K39" s="22">
         <f>SUM(K8:K38)</f>
         <v>0</v>
       </c>
-      <c r="L39" s="29"/>
-      <c r="M39" s="29">
+      <c r="L39" s="22"/>
+      <c r="M39" s="22">
         <f>SUM(M8:M38)</f>
         <v>0</v>
       </c>
-      <c r="N39" s="29"/>
-      <c r="O39" s="38">
+      <c r="N39" s="22"/>
+      <c r="O39" s="27">
         <f>SUM(O8:O38)</f>
         <v>0</v>
       </c>
-      <c r="P39" s="87" t="s">
+      <c r="P39" s="80" t="s">
         <v>8</v>
       </c>
-      <c r="Q39" s="88"/>
-      <c r="R39" s="88"/>
-      <c r="S39" s="88"/>
-      <c r="T39" s="89"/>
-      <c r="U39" s="30"/>
-      <c r="V39" s="30"/>
-      <c r="W39" s="40">
+      <c r="Q39" s="81"/>
+      <c r="R39" s="81"/>
+      <c r="S39" s="81"/>
+      <c r="T39" s="82"/>
+      <c r="U39" s="23"/>
+      <c r="V39" s="23"/>
+      <c r="W39" s="29">
         <f>SUM(W8:W38)</f>
         <v>0</v>
       </c>
-      <c r="X39" s="39">
+      <c r="X39" s="28">
         <f>SUM(X8:X38)</f>
         <v>0</v>
       </c>
-      <c r="Y39" s="90"/>
-      <c r="Z39" s="91"/>
-      <c r="AA39" s="91"/>
-      <c r="AB39" s="91"/>
-      <c r="AC39" s="91"/>
-      <c r="AD39" s="91"/>
-      <c r="AE39" s="92"/>
+      <c r="Y39" s="83"/>
+      <c r="Z39" s="84"/>
+      <c r="AA39" s="84"/>
+      <c r="AB39" s="84"/>
+      <c r="AC39" s="84"/>
+      <c r="AD39" s="84"/>
+      <c r="AE39" s="85"/>
     </row>
     <row r="40" spans="1:32">
       <c r="E40" s="3"/>
@@ -4865,14 +4636,14 @@
       <c r="A41" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="B41" s="62" t="s">
+      <c r="B41" s="36" t="s">
         <v>18</v>
       </c>
-      <c r="C41" s="63"/>
-      <c r="D41" s="63"/>
-      <c r="E41" s="63"/>
-      <c r="F41" s="63"/>
-      <c r="G41" s="63"/>
+      <c r="C41" s="37"/>
+      <c r="D41" s="37"/>
+      <c r="E41" s="37"/>
+      <c r="F41" s="37"/>
+      <c r="G41" s="37"/>
     </row>
     <row r="42" spans="1:32" ht="18" customHeight="1">
       <c r="A42" s="16" t="s">
@@ -4899,50 +4670,16 @@
       </c>
     </row>
     <row r="46" spans="1:32">
-      <c r="A46" s="93" t="s">
+      <c r="A46" s="86" t="s">
         <v>15</v>
       </c>
-      <c r="B46" s="93"/>
+      <c r="B46" s="86"/>
       <c r="C46" s="14">
         <v>0.33333333333333331</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="50">
-    <mergeCell ref="Y35:AD35"/>
-    <mergeCell ref="Y36:AD36"/>
-    <mergeCell ref="Y37:AD37"/>
-    <mergeCell ref="Y38:AD38"/>
-    <mergeCell ref="Y29:AD29"/>
-    <mergeCell ref="Y30:AD30"/>
-    <mergeCell ref="Y31:AD31"/>
-    <mergeCell ref="Y32:AD32"/>
-    <mergeCell ref="Y33:AD33"/>
-    <mergeCell ref="Y21:AD21"/>
-    <mergeCell ref="Y22:AD22"/>
-    <mergeCell ref="Y34:AD34"/>
-    <mergeCell ref="Y23:AD23"/>
-    <mergeCell ref="Y24:AD24"/>
-    <mergeCell ref="Y25:AD25"/>
-    <mergeCell ref="Y26:AD26"/>
-    <mergeCell ref="Y27:AD27"/>
-    <mergeCell ref="Y28:AD28"/>
-    <mergeCell ref="AA2:AE2"/>
-    <mergeCell ref="P2:X2"/>
-    <mergeCell ref="Y8:AD8"/>
-    <mergeCell ref="Y9:AD9"/>
-    <mergeCell ref="Y10:AD10"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A6:B7"/>
-    <mergeCell ref="C6:G6"/>
-    <mergeCell ref="K6:O6"/>
-    <mergeCell ref="P6:W6"/>
-    <mergeCell ref="AA3:AE3"/>
-    <mergeCell ref="P3:X3"/>
-    <mergeCell ref="P4:X4"/>
-    <mergeCell ref="Y6:AD7"/>
-    <mergeCell ref="AE6:AE7"/>
-    <mergeCell ref="X6:X7"/>
     <mergeCell ref="A39:B39"/>
     <mergeCell ref="P39:T39"/>
     <mergeCell ref="Y39:AE39"/>
@@ -4959,6 +4696,40 @@
     <mergeCell ref="Y18:AD18"/>
     <mergeCell ref="Y19:AD19"/>
     <mergeCell ref="Y20:AD20"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A6:B7"/>
+    <mergeCell ref="C6:G6"/>
+    <mergeCell ref="K6:O6"/>
+    <mergeCell ref="P6:W6"/>
+    <mergeCell ref="P3:X3"/>
+    <mergeCell ref="P4:X4"/>
+    <mergeCell ref="X6:X7"/>
+    <mergeCell ref="AA2:AE2"/>
+    <mergeCell ref="P2:X2"/>
+    <mergeCell ref="Y8:AD8"/>
+    <mergeCell ref="Y9:AD9"/>
+    <mergeCell ref="Y10:AD10"/>
+    <mergeCell ref="AA3:AE3"/>
+    <mergeCell ref="Y6:AD7"/>
+    <mergeCell ref="AE6:AE7"/>
+    <mergeCell ref="Y21:AD21"/>
+    <mergeCell ref="Y22:AD22"/>
+    <mergeCell ref="Y34:AD34"/>
+    <mergeCell ref="Y23:AD23"/>
+    <mergeCell ref="Y24:AD24"/>
+    <mergeCell ref="Y25:AD25"/>
+    <mergeCell ref="Y26:AD26"/>
+    <mergeCell ref="Y27:AD27"/>
+    <mergeCell ref="Y28:AD28"/>
+    <mergeCell ref="Y35:AD35"/>
+    <mergeCell ref="Y36:AD36"/>
+    <mergeCell ref="Y37:AD37"/>
+    <mergeCell ref="Y38:AD38"/>
+    <mergeCell ref="Y29:AD29"/>
+    <mergeCell ref="Y30:AD30"/>
+    <mergeCell ref="Y31:AD31"/>
+    <mergeCell ref="Y32:AD32"/>
+    <mergeCell ref="Y33:AD33"/>
   </mergeCells>
   <phoneticPr fontId="2"/>
   <dataValidations count="1">

</xml_diff>